<commit_message>
feat(saff-study): publish specification and test suite v1.7
</commit_message>
<xml_diff>
--- a/output/xlsx/CRUDCliente--GT-.xlsx
+++ b/output/xlsx/CRUDCliente--GT-.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="249" uniqueCount="51">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="321" uniqueCount="55">
   <si>
     <t xml:space="preserve">System: </t>
   </si>
@@ -38,7 +38,7 @@
     <t>Reduced (Greedy Heuristic - Transition Coverage)</t>
   </si>
   <si>
-    <t>Size: 4 test case(s)</t>
+    <t>Size: 5 test case(s)</t>
   </si>
   <si>
     <t xml:space="preserve">Creation Date: </t>
@@ -92,7 +92,7 @@
     <t>Actual Result</t>
   </si>
   <si>
-    <t>superAdmin: seleciona opção 'Customers' no menu Settings</t>
+    <t>superAdmin: seleciona opcao 'Customers' no menu Settings</t>
   </si>
   <si>
     <t/>
@@ -104,13 +104,13 @@
     <t>superAdmin: seleciona o botão 'Create Customer'</t>
   </si>
   <si>
-    <t>SYSTEM exibe página com campos de cadastro de novo cliente</t>
-  </si>
-  <si>
-    <t xml:space="preserve">superAdmin: preenche corretamente os campos 'Name', 'Key File' e 'Country' e pressiona o botão 'Create' </t>
-  </si>
-  <si>
-    <t>SYSTEM exibe página com dados do novo cliente e mensagem que um novo cliente foi adicionado</t>
+    <t>SYSTEM exibe pagina com campos de cadastro de novo cliente</t>
+  </si>
+  <si>
+    <t xml:space="preserve">superAdmin: preenche corretamente os campos 'Name', 'Key File' e 'Country' e pressiona o botao 'Create' </t>
+  </si>
+  <si>
+    <t>SYSTEM exibe pagina com dados do novo cliente e mensagem que um novo cliente foi adicionado</t>
   </si>
   <si>
     <t>superAdmin: clica no nome de um cliente</t>
@@ -119,7 +119,7 @@
     <t>SYSTEM exibe dados do cliente</t>
   </si>
   <si>
-    <t>superAdmin: clica no botão 'Cancel'</t>
+    <t>superAdmin: clica no botao 'Cancel'</t>
   </si>
   <si>
     <t>SYSTEM retorna a lista de clientes</t>
@@ -131,40 +131,52 @@
     <t>TC2</t>
   </si>
   <si>
-    <t>Alternative Flow 1: Cancela criação</t>
-  </si>
-  <si>
-    <t>superAdmin: Cancela criação</t>
+    <t>Alternative Flow 1: Campo fora da formatacao esperada, e.g., 'ddd' para 'Key File'</t>
+  </si>
+  <si>
+    <t xml:space="preserve">superAdmin: preenche incorretamente os campos 'Name', 'Key File' e/ou 'Country' e pressiona o botão 'Create' </t>
+  </si>
+  <si>
+    <t>SYSTEM exibe mensagem informando que os dados nao correspondem a formatação esperada</t>
   </si>
   <si>
     <t>TC3</t>
   </si>
   <si>
-    <t>Alternative Flow 2: Edita dados</t>
-  </si>
-  <si>
-    <t>superAdmin: clica no botão 'Edit'</t>
+    <t>Alternative Flow 2: Cancela criacao</t>
+  </si>
+  <si>
+    <t>superAdmin: Cancela criacao</t>
+  </si>
+  <si>
+    <t>TC4</t>
+  </si>
+  <si>
+    <t>Alternative Flow 3: Edita dados</t>
+  </si>
+  <si>
+    <t>superAdmin: clica no botao 'Edit'</t>
   </si>
   <si>
     <t>SYSTEM exibe campos do cliente com valores atuais que podem ser editados</t>
   </si>
   <si>
-    <t>superAdmin: preenche os novos valores e pressiona o botão 'Update</t>
-  </si>
-  <si>
-    <t>TC4</t>
-  </si>
-  <si>
-    <t>Alternative Flow 3: Deleta cliente</t>
-  </si>
-  <si>
-    <t>superAdmin: clica no botão 'Delete'</t>
-  </si>
-  <si>
-    <t>SYSTEM exibe mensagem solicitando confirmação</t>
-  </si>
-  <si>
-    <t>superAdmin: pressiona o botão OK</t>
+    <t>superAdmin: preenche os novos valores e pressiona o botao 'Update</t>
+  </si>
+  <si>
+    <t>TC5</t>
+  </si>
+  <si>
+    <t>Alternative Flow 4: Deleta cliente</t>
+  </si>
+  <si>
+    <t>superAdmin: clica no botao 'Delete'</t>
+  </si>
+  <si>
+    <t>SYSTEM exibe mensagem solicitando confirmacao</t>
+  </si>
+  <si>
+    <t>superAdmin: pressiona o botao OK</t>
   </si>
 </sst>
 </file>
@@ -256,11 +268,11 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:F65"/>
+  <dimension ref="A1:F83"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
   <cols>
     <col min="1" max="1" width="17.578125" customWidth="true" bestFit="true"/>
-    <col min="2" max="2" width="86.19140625" customWidth="true" bestFit="true"/>
+    <col min="2" max="2" width="90.51953125" customWidth="true" bestFit="true"/>
     <col min="3" max="3" width="21.8984375" customWidth="true" bestFit="true"/>
     <col min="4" max="4" width="79.19921875" customWidth="true" bestFit="true"/>
     <col min="5" max="5" width="30.5234375" customWidth="true" bestFit="true"/>
@@ -591,7 +603,7 @@
         <v>27</v>
       </c>
       <c r="D25" t="s" s="3">
-        <v>28</v>
+        <v>41</v>
       </c>
       <c r="E25" t="s" s="3">
         <v>27</v>
@@ -605,13 +617,13 @@
         <v>4.0</v>
       </c>
       <c r="B26" t="s" s="3">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="C26" t="s" s="3">
         <v>27</v>
       </c>
       <c r="D26" t="s" s="3">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="E26" t="s" s="3">
         <v>27</v>
@@ -625,13 +637,13 @@
         <v>5.0</v>
       </c>
       <c r="B27" t="s" s="3">
-        <v>31</v>
+        <v>26</v>
       </c>
       <c r="C27" t="s" s="3">
         <v>27</v>
       </c>
       <c r="D27" t="s" s="3">
-        <v>32</v>
+        <v>28</v>
       </c>
       <c r="E27" t="s" s="3">
         <v>27</v>
@@ -645,13 +657,13 @@
         <v>6.0</v>
       </c>
       <c r="B28" t="s" s="3">
-        <v>26</v>
+        <v>33</v>
       </c>
       <c r="C28" t="s" s="3">
         <v>27</v>
       </c>
       <c r="D28" t="s" s="3">
-        <v>28</v>
+        <v>34</v>
       </c>
       <c r="E28" t="s" s="3">
         <v>27</v>
@@ -665,13 +677,13 @@
         <v>7.0</v>
       </c>
       <c r="B29" t="s" s="3">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="C29" t="s" s="3">
         <v>27</v>
       </c>
       <c r="D29" t="s" s="3">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="E29" t="s" s="3">
         <v>27</v>
@@ -681,98 +693,98 @@
       </c>
     </row>
     <row r="30">
-      <c r="A30" t="n" s="4">
-        <v>8.0</v>
-      </c>
-      <c r="B30" t="s" s="3">
-        <v>35</v>
-      </c>
-      <c r="C30" t="s" s="3">
-        <v>27</v>
-      </c>
-      <c r="D30" t="s" s="3">
-        <v>36</v>
-      </c>
-      <c r="E30" t="s" s="3">
-        <v>27</v>
-      </c>
-      <c r="F30" t="s" s="3">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="31">
-      <c r="A31" t="s" s="1">
+      <c r="A30" t="s" s="1">
         <v>37</v>
       </c>
-      <c r="B31" t="s" s="0">
-        <v>27</v>
+      <c r="B30" t="s" s="0">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="s" s="1">
+        <v>11</v>
+      </c>
+      <c r="B33" t="s" s="0">
+        <v>42</v>
+      </c>
+      <c r="C33" t="s" s="1">
+        <v>13</v>
+      </c>
+      <c r="E33" t="s" s="1">
+        <v>14</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="s" s="1">
-        <v>11</v>
+        <v>15</v>
       </c>
       <c r="B34" t="s" s="0">
-        <v>41</v>
-      </c>
-      <c r="C34" t="s" s="1">
-        <v>13</v>
+        <v>43</v>
       </c>
       <c r="E34" t="s" s="1">
-        <v>14</v>
+        <v>17</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="s" s="1">
-        <v>15</v>
+        <v>18</v>
       </c>
       <c r="B35" t="s" s="0">
-        <v>42</v>
-      </c>
-      <c r="E35" t="s" s="1">
-        <v>17</v>
+        <v>19</v>
       </c>
     </row>
     <row r="36">
-      <c r="A36" t="s" s="1">
-        <v>18</v>
-      </c>
-      <c r="B36" t="s" s="0">
-        <v>19</v>
+      <c r="A36" t="s" s="2">
+        <v>20</v>
+      </c>
+      <c r="B36" t="s" s="2">
+        <v>21</v>
+      </c>
+      <c r="C36" t="s" s="2">
+        <v>22</v>
+      </c>
+      <c r="D36" t="s" s="2">
+        <v>23</v>
+      </c>
+      <c r="E36" t="s" s="2">
+        <v>24</v>
+      </c>
+      <c r="F36" t="s" s="2">
+        <v>25</v>
       </c>
     </row>
     <row r="37">
-      <c r="A37" t="s" s="2">
-        <v>20</v>
-      </c>
-      <c r="B37" t="s" s="2">
-        <v>21</v>
-      </c>
-      <c r="C37" t="s" s="2">
-        <v>22</v>
-      </c>
-      <c r="D37" t="s" s="2">
-        <v>23</v>
-      </c>
-      <c r="E37" t="s" s="2">
-        <v>24</v>
-      </c>
-      <c r="F37" t="s" s="2">
-        <v>25</v>
+      <c r="A37" t="n" s="4">
+        <v>1.0</v>
+      </c>
+      <c r="B37" t="s" s="3">
+        <v>26</v>
+      </c>
+      <c r="C37" t="s" s="3">
+        <v>27</v>
+      </c>
+      <c r="D37" t="s" s="3">
+        <v>28</v>
+      </c>
+      <c r="E37" t="s" s="3">
+        <v>27</v>
+      </c>
+      <c r="F37" t="s" s="3">
+        <v>27</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="n" s="4">
-        <v>1.0</v>
+        <v>2.0</v>
       </c>
       <c r="B38" t="s" s="3">
-        <v>26</v>
+        <v>29</v>
       </c>
       <c r="C38" t="s" s="3">
         <v>27</v>
       </c>
       <c r="D38" t="s" s="3">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="E38" t="s" s="3">
         <v>27</v>
@@ -783,16 +795,16 @@
     </row>
     <row r="39">
       <c r="A39" t="n" s="4">
-        <v>2.0</v>
+        <v>3.0</v>
       </c>
       <c r="B39" t="s" s="3">
-        <v>29</v>
+        <v>44</v>
       </c>
       <c r="C39" t="s" s="3">
         <v>27</v>
       </c>
       <c r="D39" t="s" s="3">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="E39" t="s" s="3">
         <v>27</v>
@@ -803,16 +815,16 @@
     </row>
     <row r="40">
       <c r="A40" t="n" s="4">
-        <v>3.0</v>
+        <v>4.0</v>
       </c>
       <c r="B40" t="s" s="3">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="C40" t="s" s="3">
         <v>27</v>
       </c>
       <c r="D40" t="s" s="3">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="E40" t="s" s="3">
         <v>27</v>
@@ -823,16 +835,16 @@
     </row>
     <row r="41">
       <c r="A41" t="n" s="4">
-        <v>4.0</v>
+        <v>5.0</v>
       </c>
       <c r="B41" t="s" s="3">
-        <v>26</v>
+        <v>31</v>
       </c>
       <c r="C41" t="s" s="3">
         <v>27</v>
       </c>
       <c r="D41" t="s" s="3">
-        <v>28</v>
+        <v>32</v>
       </c>
       <c r="E41" t="s" s="3">
         <v>27</v>
@@ -843,16 +855,16 @@
     </row>
     <row r="42">
       <c r="A42" t="n" s="4">
-        <v>5.0</v>
+        <v>6.0</v>
       </c>
       <c r="B42" t="s" s="3">
-        <v>33</v>
+        <v>26</v>
       </c>
       <c r="C42" t="s" s="3">
         <v>27</v>
       </c>
       <c r="D42" t="s" s="3">
-        <v>34</v>
+        <v>28</v>
       </c>
       <c r="E42" t="s" s="3">
         <v>27</v>
@@ -863,16 +875,16 @@
     </row>
     <row r="43">
       <c r="A43" t="n" s="4">
-        <v>6.0</v>
+        <v>7.0</v>
       </c>
       <c r="B43" t="s" s="3">
-        <v>43</v>
+        <v>33</v>
       </c>
       <c r="C43" t="s" s="3">
         <v>27</v>
       </c>
       <c r="D43" t="s" s="3">
-        <v>44</v>
+        <v>34</v>
       </c>
       <c r="E43" t="s" s="3">
         <v>27</v>
@@ -883,117 +895,117 @@
     </row>
     <row r="44">
       <c r="A44" t="n" s="4">
-        <v>7.0</v>
+        <v>8.0</v>
       </c>
       <c r="B44" t="s" s="3">
+        <v>35</v>
+      </c>
+      <c r="C44" t="s" s="3">
+        <v>27</v>
+      </c>
+      <c r="D44" t="s" s="3">
+        <v>36</v>
+      </c>
+      <c r="E44" t="s" s="3">
+        <v>27</v>
+      </c>
+      <c r="F44" t="s" s="3">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="s" s="1">
+        <v>37</v>
+      </c>
+      <c r="B45" t="s" s="0">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="s" s="1">
+        <v>11</v>
+      </c>
+      <c r="B48" t="s" s="0">
         <v>45</v>
       </c>
-      <c r="C44" t="s" s="3">
-        <v>27</v>
-      </c>
-      <c r="D44" t="s" s="3">
-        <v>34</v>
-      </c>
-      <c r="E44" t="s" s="3">
-        <v>27</v>
-      </c>
-      <c r="F44" t="s" s="3">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="45">
-      <c r="A45" t="n" s="4">
-        <v>8.0</v>
-      </c>
-      <c r="B45" t="s" s="3">
-        <v>35</v>
-      </c>
-      <c r="C45" t="s" s="3">
-        <v>27</v>
-      </c>
-      <c r="D45" t="s" s="3">
-        <v>36</v>
-      </c>
-      <c r="E45" t="s" s="3">
-        <v>27</v>
-      </c>
-      <c r="F45" t="s" s="3">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="46">
-      <c r="A46" t="s" s="1">
-        <v>37</v>
-      </c>
-      <c r="B46" t="s" s="0">
-        <v>27</v>
+      <c r="C48" t="s" s="1">
+        <v>13</v>
+      </c>
+      <c r="E48" t="s" s="1">
+        <v>14</v>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="s" s="1">
-        <v>11</v>
+        <v>15</v>
       </c>
       <c r="B49" t="s" s="0">
         <v>46</v>
       </c>
-      <c r="C49" t="s" s="1">
-        <v>13</v>
-      </c>
       <c r="E49" t="s" s="1">
-        <v>14</v>
+        <v>17</v>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="s" s="1">
-        <v>15</v>
+        <v>18</v>
       </c>
       <c r="B50" t="s" s="0">
-        <v>47</v>
-      </c>
-      <c r="E50" t="s" s="1">
-        <v>17</v>
+        <v>19</v>
       </c>
     </row>
     <row r="51">
-      <c r="A51" t="s" s="1">
-        <v>18</v>
-      </c>
-      <c r="B51" t="s" s="0">
-        <v>19</v>
+      <c r="A51" t="s" s="2">
+        <v>20</v>
+      </c>
+      <c r="B51" t="s" s="2">
+        <v>21</v>
+      </c>
+      <c r="C51" t="s" s="2">
+        <v>22</v>
+      </c>
+      <c r="D51" t="s" s="2">
+        <v>23</v>
+      </c>
+      <c r="E51" t="s" s="2">
+        <v>24</v>
+      </c>
+      <c r="F51" t="s" s="2">
+        <v>25</v>
       </c>
     </row>
     <row r="52">
-      <c r="A52" t="s" s="2">
-        <v>20</v>
-      </c>
-      <c r="B52" t="s" s="2">
-        <v>21</v>
-      </c>
-      <c r="C52" t="s" s="2">
-        <v>22</v>
-      </c>
-      <c r="D52" t="s" s="2">
-        <v>23</v>
-      </c>
-      <c r="E52" t="s" s="2">
-        <v>24</v>
-      </c>
-      <c r="F52" t="s" s="2">
-        <v>25</v>
+      <c r="A52" t="n" s="4">
+        <v>1.0</v>
+      </c>
+      <c r="B52" t="s" s="3">
+        <v>26</v>
+      </c>
+      <c r="C52" t="s" s="3">
+        <v>27</v>
+      </c>
+      <c r="D52" t="s" s="3">
+        <v>28</v>
+      </c>
+      <c r="E52" t="s" s="3">
+        <v>27</v>
+      </c>
+      <c r="F52" t="s" s="3">
+        <v>27</v>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="n" s="4">
-        <v>1.0</v>
+        <v>2.0</v>
       </c>
       <c r="B53" t="s" s="3">
-        <v>26</v>
+        <v>29</v>
       </c>
       <c r="C53" t="s" s="3">
         <v>27</v>
       </c>
       <c r="D53" t="s" s="3">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="E53" t="s" s="3">
         <v>27</v>
@@ -1004,16 +1016,16 @@
     </row>
     <row r="54">
       <c r="A54" t="n" s="4">
-        <v>2.0</v>
+        <v>3.0</v>
       </c>
       <c r="B54" t="s" s="3">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="C54" t="s" s="3">
         <v>27</v>
       </c>
       <c r="D54" t="s" s="3">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="E54" t="s" s="3">
         <v>27</v>
@@ -1024,16 +1036,16 @@
     </row>
     <row r="55">
       <c r="A55" t="n" s="4">
-        <v>3.0</v>
+        <v>4.0</v>
       </c>
       <c r="B55" t="s" s="3">
-        <v>31</v>
+        <v>26</v>
       </c>
       <c r="C55" t="s" s="3">
         <v>27</v>
       </c>
       <c r="D55" t="s" s="3">
-        <v>32</v>
+        <v>28</v>
       </c>
       <c r="E55" t="s" s="3">
         <v>27</v>
@@ -1044,16 +1056,16 @@
     </row>
     <row r="56">
       <c r="A56" t="n" s="4">
-        <v>4.0</v>
+        <v>5.0</v>
       </c>
       <c r="B56" t="s" s="3">
-        <v>26</v>
+        <v>33</v>
       </c>
       <c r="C56" t="s" s="3">
         <v>27</v>
       </c>
       <c r="D56" t="s" s="3">
-        <v>28</v>
+        <v>34</v>
       </c>
       <c r="E56" t="s" s="3">
         <v>27</v>
@@ -1064,16 +1076,16 @@
     </row>
     <row r="57">
       <c r="A57" t="n" s="4">
-        <v>5.0</v>
+        <v>6.0</v>
       </c>
       <c r="B57" t="s" s="3">
-        <v>33</v>
+        <v>47</v>
       </c>
       <c r="C57" t="s" s="3">
         <v>27</v>
       </c>
       <c r="D57" t="s" s="3">
-        <v>34</v>
+        <v>48</v>
       </c>
       <c r="E57" t="s" s="3">
         <v>27</v>
@@ -1084,16 +1096,16 @@
     </row>
     <row r="58">
       <c r="A58" t="n" s="4">
-        <v>6.0</v>
+        <v>7.0</v>
       </c>
       <c r="B58" t="s" s="3">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="C58" t="s" s="3">
         <v>27</v>
       </c>
       <c r="D58" t="s" s="3">
-        <v>49</v>
+        <v>28</v>
       </c>
       <c r="E58" t="s" s="3">
         <v>27</v>
@@ -1104,16 +1116,16 @@
     </row>
     <row r="59">
       <c r="A59" t="n" s="4">
-        <v>7.0</v>
+        <v>8.0</v>
       </c>
       <c r="B59" t="s" s="3">
-        <v>50</v>
+        <v>29</v>
       </c>
       <c r="C59" t="s" s="3">
         <v>27</v>
       </c>
       <c r="D59" t="s" s="3">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="E59" t="s" s="3">
         <v>27</v>
@@ -1124,16 +1136,16 @@
     </row>
     <row r="60">
       <c r="A60" t="n" s="4">
-        <v>8.0</v>
+        <v>9.0</v>
       </c>
       <c r="B60" t="s" s="3">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="C60" t="s" s="3">
         <v>27</v>
       </c>
       <c r="D60" t="s" s="3">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="E60" t="s" s="3">
         <v>27</v>
@@ -1144,16 +1156,16 @@
     </row>
     <row r="61">
       <c r="A61" t="n" s="4">
-        <v>9.0</v>
+        <v>10.0</v>
       </c>
       <c r="B61" t="s" s="3">
-        <v>31</v>
+        <v>26</v>
       </c>
       <c r="C61" t="s" s="3">
         <v>27</v>
       </c>
       <c r="D61" t="s" s="3">
-        <v>32</v>
+        <v>28</v>
       </c>
       <c r="E61" t="s" s="3">
         <v>27</v>
@@ -1164,16 +1176,16 @@
     </row>
     <row r="62">
       <c r="A62" t="n" s="4">
-        <v>10.0</v>
+        <v>11.0</v>
       </c>
       <c r="B62" t="s" s="3">
-        <v>26</v>
+        <v>33</v>
       </c>
       <c r="C62" t="s" s="3">
         <v>27</v>
       </c>
       <c r="D62" t="s" s="3">
-        <v>28</v>
+        <v>34</v>
       </c>
       <c r="E62" t="s" s="3">
         <v>27</v>
@@ -1184,49 +1196,330 @@
     </row>
     <row r="63">
       <c r="A63" t="n" s="4">
+        <v>12.0</v>
+      </c>
+      <c r="B63" t="s" s="3">
+        <v>35</v>
+      </c>
+      <c r="C63" t="s" s="3">
+        <v>27</v>
+      </c>
+      <c r="D63" t="s" s="3">
+        <v>36</v>
+      </c>
+      <c r="E63" t="s" s="3">
+        <v>27</v>
+      </c>
+      <c r="F63" t="s" s="3">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="s" s="1">
+        <v>37</v>
+      </c>
+      <c r="B64" t="s" s="0">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="s" s="1">
+        <v>11</v>
+      </c>
+      <c r="B67" t="s" s="0">
+        <v>50</v>
+      </c>
+      <c r="C67" t="s" s="1">
+        <v>13</v>
+      </c>
+      <c r="E67" t="s" s="1">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="s" s="1">
+        <v>15</v>
+      </c>
+      <c r="B68" t="s" s="0">
+        <v>51</v>
+      </c>
+      <c r="E68" t="s" s="1">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="s" s="1">
+        <v>18</v>
+      </c>
+      <c r="B69" t="s" s="0">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="s" s="2">
+        <v>20</v>
+      </c>
+      <c r="B70" t="s" s="2">
+        <v>21</v>
+      </c>
+      <c r="C70" t="s" s="2">
+        <v>22</v>
+      </c>
+      <c r="D70" t="s" s="2">
+        <v>23</v>
+      </c>
+      <c r="E70" t="s" s="2">
+        <v>24</v>
+      </c>
+      <c r="F70" t="s" s="2">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="n" s="4">
+        <v>1.0</v>
+      </c>
+      <c r="B71" t="s" s="3">
+        <v>26</v>
+      </c>
+      <c r="C71" t="s" s="3">
+        <v>27</v>
+      </c>
+      <c r="D71" t="s" s="3">
+        <v>28</v>
+      </c>
+      <c r="E71" t="s" s="3">
+        <v>27</v>
+      </c>
+      <c r="F71" t="s" s="3">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="n" s="4">
+        <v>2.0</v>
+      </c>
+      <c r="B72" t="s" s="3">
+        <v>29</v>
+      </c>
+      <c r="C72" t="s" s="3">
+        <v>27</v>
+      </c>
+      <c r="D72" t="s" s="3">
+        <v>30</v>
+      </c>
+      <c r="E72" t="s" s="3">
+        <v>27</v>
+      </c>
+      <c r="F72" t="s" s="3">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="n" s="4">
+        <v>3.0</v>
+      </c>
+      <c r="B73" t="s" s="3">
+        <v>31</v>
+      </c>
+      <c r="C73" t="s" s="3">
+        <v>27</v>
+      </c>
+      <c r="D73" t="s" s="3">
+        <v>32</v>
+      </c>
+      <c r="E73" t="s" s="3">
+        <v>27</v>
+      </c>
+      <c r="F73" t="s" s="3">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" t="n" s="4">
+        <v>4.0</v>
+      </c>
+      <c r="B74" t="s" s="3">
+        <v>26</v>
+      </c>
+      <c r="C74" t="s" s="3">
+        <v>27</v>
+      </c>
+      <c r="D74" t="s" s="3">
+        <v>28</v>
+      </c>
+      <c r="E74" t="s" s="3">
+        <v>27</v>
+      </c>
+      <c r="F74" t="s" s="3">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" t="n" s="4">
+        <v>5.0</v>
+      </c>
+      <c r="B75" t="s" s="3">
+        <v>33</v>
+      </c>
+      <c r="C75" t="s" s="3">
+        <v>27</v>
+      </c>
+      <c r="D75" t="s" s="3">
+        <v>34</v>
+      </c>
+      <c r="E75" t="s" s="3">
+        <v>27</v>
+      </c>
+      <c r="F75" t="s" s="3">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" t="n" s="4">
+        <v>6.0</v>
+      </c>
+      <c r="B76" t="s" s="3">
+        <v>52</v>
+      </c>
+      <c r="C76" t="s" s="3">
+        <v>27</v>
+      </c>
+      <c r="D76" t="s" s="3">
+        <v>53</v>
+      </c>
+      <c r="E76" t="s" s="3">
+        <v>27</v>
+      </c>
+      <c r="F76" t="s" s="3">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" t="n" s="4">
+        <v>7.0</v>
+      </c>
+      <c r="B77" t="s" s="3">
+        <v>54</v>
+      </c>
+      <c r="C77" t="s" s="3">
+        <v>27</v>
+      </c>
+      <c r="D77" t="s" s="3">
+        <v>28</v>
+      </c>
+      <c r="E77" t="s" s="3">
+        <v>27</v>
+      </c>
+      <c r="F77" t="s" s="3">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" t="n" s="4">
+        <v>8.0</v>
+      </c>
+      <c r="B78" t="s" s="3">
+        <v>29</v>
+      </c>
+      <c r="C78" t="s" s="3">
+        <v>27</v>
+      </c>
+      <c r="D78" t="s" s="3">
+        <v>30</v>
+      </c>
+      <c r="E78" t="s" s="3">
+        <v>27</v>
+      </c>
+      <c r="F78" t="s" s="3">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" t="n" s="4">
+        <v>9.0</v>
+      </c>
+      <c r="B79" t="s" s="3">
+        <v>31</v>
+      </c>
+      <c r="C79" t="s" s="3">
+        <v>27</v>
+      </c>
+      <c r="D79" t="s" s="3">
+        <v>32</v>
+      </c>
+      <c r="E79" t="s" s="3">
+        <v>27</v>
+      </c>
+      <c r="F79" t="s" s="3">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" t="n" s="4">
+        <v>10.0</v>
+      </c>
+      <c r="B80" t="s" s="3">
+        <v>26</v>
+      </c>
+      <c r="C80" t="s" s="3">
+        <v>27</v>
+      </c>
+      <c r="D80" t="s" s="3">
+        <v>28</v>
+      </c>
+      <c r="E80" t="s" s="3">
+        <v>27</v>
+      </c>
+      <c r="F80" t="s" s="3">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" t="n" s="4">
         <v>11.0</v>
       </c>
-      <c r="B63" t="s" s="3">
+      <c r="B81" t="s" s="3">
         <v>33</v>
       </c>
-      <c r="C63" t="s" s="3">
-        <v>27</v>
-      </c>
-      <c r="D63" t="s" s="3">
+      <c r="C81" t="s" s="3">
+        <v>27</v>
+      </c>
+      <c r="D81" t="s" s="3">
         <v>34</v>
       </c>
-      <c r="E63" t="s" s="3">
-        <v>27</v>
-      </c>
-      <c r="F63" t="s" s="3">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="64">
-      <c r="A64" t="n" s="4">
+      <c r="E81" t="s" s="3">
+        <v>27</v>
+      </c>
+      <c r="F81" t="s" s="3">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" t="n" s="4">
         <v>12.0</v>
       </c>
-      <c r="B64" t="s" s="3">
+      <c r="B82" t="s" s="3">
         <v>35</v>
       </c>
-      <c r="C64" t="s" s="3">
-        <v>27</v>
-      </c>
-      <c r="D64" t="s" s="3">
+      <c r="C82" t="s" s="3">
+        <v>27</v>
+      </c>
+      <c r="D82" t="s" s="3">
         <v>36</v>
       </c>
-      <c r="E64" t="s" s="3">
-        <v>27</v>
-      </c>
-      <c r="F64" t="s" s="3">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="65">
-      <c r="A65" t="s" s="1">
+      <c r="E82" t="s" s="3">
+        <v>27</v>
+      </c>
+      <c r="F82" t="s" s="3">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" t="s" s="1">
         <v>37</v>
       </c>
-      <c r="B65" t="s" s="0">
+      <c r="B83" t="s" s="0">
         <v>27</v>
       </c>
     </row>

</xml_diff>

<commit_message>
feat(saff-study): publish specification and test suite v1.8
</commit_message>
<xml_diff>
--- a/output/xlsx/CRUDCliente--GT-.xlsx
+++ b/output/xlsx/CRUDCliente--GT-.xlsx
@@ -92,7 +92,7 @@
     <t>Actual Result</t>
   </si>
   <si>
-    <t>superAdmin: seleciona opcao 'Customers' no menu Settings</t>
+    <t>superAdmin: seleciona opção 'Customers' no menu Settings</t>
   </si>
   <si>
     <t/>
@@ -104,13 +104,13 @@
     <t>superAdmin: seleciona o botão 'Create Customer'</t>
   </si>
   <si>
-    <t>SYSTEM exibe pagina com campos de cadastro de novo cliente</t>
-  </si>
-  <si>
-    <t xml:space="preserve">superAdmin: preenche corretamente os campos 'Name', 'Key File' e 'Country' e pressiona o botao 'Create' </t>
-  </si>
-  <si>
-    <t>SYSTEM exibe pagina com dados do novo cliente e mensagem que um novo cliente foi adicionado</t>
+    <t>SYSTEM exibe página com campos de cadastro de novo cliente</t>
+  </si>
+  <si>
+    <t xml:space="preserve">superAdmin: preenche corretamente os campos 'Name', 'Key File' e 'Country' e pressiona o botão 'Create' </t>
+  </si>
+  <si>
+    <t>SYSTEM exibe página com dados do novo cliente e mensagem que um novo cliente foi adicionado</t>
   </si>
   <si>
     <t>superAdmin: clica no nome de um cliente</t>
@@ -119,7 +119,7 @@
     <t>SYSTEM exibe dados do cliente</t>
   </si>
   <si>
-    <t>superAdmin: clica no botao 'Cancel'</t>
+    <t>superAdmin: clica no botão 'Cancel'</t>
   </si>
   <si>
     <t>SYSTEM retorna a lista de clientes</t>
@@ -131,22 +131,22 @@
     <t>TC2</t>
   </si>
   <si>
-    <t>Alternative Flow 1: Campo fora da formatacao esperada, e.g., 'ddd' para 'Key File'</t>
+    <t>Alternative Flow 1: Campo fora da formatação esperada, e.g., 'ddd' para 'Key File'</t>
   </si>
   <si>
     <t xml:space="preserve">superAdmin: preenche incorretamente os campos 'Name', 'Key File' e/ou 'Country' e pressiona o botão 'Create' </t>
   </si>
   <si>
-    <t>SYSTEM exibe mensagem informando que os dados nao correspondem a formatação esperada</t>
+    <t>SYSTEM exibe mensagem informando que os dados não correspondem a formatação esperada</t>
   </si>
   <si>
     <t>TC3</t>
   </si>
   <si>
-    <t>Alternative Flow 2: Cancela criacao</t>
-  </si>
-  <si>
-    <t>superAdmin: Cancela criacao</t>
+    <t>Alternative Flow 2: Cancela criação</t>
+  </si>
+  <si>
+    <t>superAdmin: Cancela criação</t>
   </si>
   <si>
     <t>TC4</t>
@@ -155,13 +155,13 @@
     <t>Alternative Flow 3: Edita dados</t>
   </si>
   <si>
-    <t>superAdmin: clica no botao 'Edit'</t>
+    <t>superAdmin: clica no botão 'Edit'</t>
   </si>
   <si>
     <t>SYSTEM exibe campos do cliente com valores atuais que podem ser editados</t>
   </si>
   <si>
-    <t>superAdmin: preenche os novos valores e pressiona o botao 'Update</t>
+    <t>superAdmin: preenche os novos valores e pressiona o botão 'Update</t>
   </si>
   <si>
     <t>TC5</t>
@@ -170,10 +170,10 @@
     <t>Alternative Flow 4: Deleta cliente</t>
   </si>
   <si>
-    <t>superAdmin: clica no botao 'Delete'</t>
-  </si>
-  <si>
-    <t>SYSTEM exibe mensagem solicitando confirmacao</t>
+    <t>superAdmin: clica no botão 'Delete'</t>
+  </si>
+  <si>
+    <t>SYSTEM exibe mensagem solicitando confirmação</t>
   </si>
   <si>
     <t>superAdmin: pressiona o botao OK</t>

</xml_diff>